<commit_message>
added excel practice files and updated project documentation
</commit_message>
<xml_diff>
--- a/Projects/Biometric Att. Data.xlsx
+++ b/Projects/Biometric Att. Data.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\mx excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Excel\Projects\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61F7EB08-D5A8-45BF-9C50-92B2A7538F08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD542DAB-4674-4D3B-94E9-C833FC51F736}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{D315C24C-E30C-44BE-AB48-08F999001083}"/>
   </bookViews>
@@ -629,6 +629,15 @@
   </cellStyles>
   <dxfs count="4">
     <dxf>
+      <numFmt numFmtId="25" formatCode="hh:mm"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="25" formatCode="hh:mm"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+    </dxf>
+    <dxf>
       <font>
         <b/>
         <i val="0"/>
@@ -651,15 +660,6 @@
           <bgColor theme="1" tint="0.499984740745262"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="25" formatCode="hh:mm"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="25" formatCode="hh:mm"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1675,7 +1675,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7944ED58-003C-420D-9CA6-EF5FB5F9F5F3}" name="Table1" displayName="Table1" ref="A1:H1051" totalsRowShown="0" headerRowDxfId="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7944ED58-003C-420D-9CA6-EF5FB5F9F5F3}" name="Table1" displayName="Table1" ref="A1:H1051" totalsRowShown="0" headerRowDxfId="3">
   <autoFilter ref="A1:H1051" xr:uid="{7944ED58-003C-420D-9CA6-EF5FB5F9F5F3}">
     <filterColumn colId="3">
       <filters>
@@ -1685,12 +1685,12 @@
   </autoFilter>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{4E746563-EB89-4C48-A5D9-97CA3318C771}" name="Emp ID "/>
-    <tableColumn id="2" xr3:uid="{F4657B0E-6135-4524-903F-22C784D55843}" name=" Date " dataDxfId="3"/>
+    <tableColumn id="2" xr3:uid="{F4657B0E-6135-4524-903F-22C784D55843}" name=" Date " dataDxfId="2"/>
     <tableColumn id="3" xr3:uid="{3A8CCE27-A6EA-4795-A387-A7C0237A08C2}" name="Full Name"/>
     <tableColumn id="4" xr3:uid="{C24D86D5-3E90-4A06-BA02-D66A7BA73043}" name="Department"/>
     <tableColumn id="5" xr3:uid="{0E5C81DE-1B95-414B-ACC6-81A8BB75AA09}" name="Designation"/>
-    <tableColumn id="6" xr3:uid="{2A95599C-9924-486C-B55C-A01897A37B44}" name=" In Time " dataDxfId="2"/>
-    <tableColumn id="7" xr3:uid="{2B27E8D9-C33B-43B1-B4E2-F42E2220E9CA}" name=" Out Time" dataDxfId="1"/>
+    <tableColumn id="6" xr3:uid="{2A95599C-9924-486C-B55C-A01897A37B44}" name=" In Time " dataDxfId="1"/>
+    <tableColumn id="7" xr3:uid="{2B27E8D9-C33B-43B1-B4E2-F42E2220E9CA}" name=" Out Time" dataDxfId="0"/>
     <tableColumn id="8" xr3:uid="{727655EF-3503-4F9E-8EBE-39C68FD26644}" name="Half/Full Day">
       <calculatedColumnFormula>IF((G2-F2)&lt;TIME(5,0,0), "Half Day", "Full Day")</calculatedColumnFormula>
     </tableColumn>

</xml_diff>